<commit_message>
Denmark 2022 results: 4,875 kt CO2e = 7.5% of the national footprint
Headline (health + eldercare, basic prices, screened v3.10.2): GWP 4,875 kt
(~0.82 t/capita; 7.5% of the model CBA of 64.7 Mt, 7.8% vs DST AFTRYK);
materials 5,595 kt (6.8%); blue water 43.0 Mm3 (4.9%); land 3,833 km2 (4.4%);
waste 1,482 kt (6.3%). Scopes 142/404/4,086/243 - Scope 2 now 8.3% of total,
matching Arup's Denmark sheet. Transport = 7.0% of GWP (11.7% of the MRIO
part): the 2016-vintage ~40% transport headline does not survive the vintage
update (see recipe_validation_2022.csv and docs/revision/analysis_2022.md).
MC: Scenario A median 4,773 [4,407-5,189]; Scenario B (pharma-specific) 3,918.
</commit_message>
<xml_diff>
--- a/data/gold/results/full_results_tables.xlsx
+++ b/data/gold/results/full_results_tables.xlsx
@@ -462,19 +462,19 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>403.7975149234967</v>
+        <v>202.3267917257008</v>
       </c>
       <c r="C2">
-        <v>112.6500772207951</v>
+        <v>206.6101087752129</v>
       </c>
       <c r="D2">
-        <v>17.53150099957248</v>
+        <v>6.51880060624706</v>
       </c>
       <c r="E2">
-        <v>1337.835798274048</v>
+        <v>581.7107327374586</v>
       </c>
       <c r="F2">
-        <v>178.327972980623</v>
+        <v>90.06703665493437</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -482,19 +482,19 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>72.53929140621092</v>
+        <v>204.9413729810275</v>
       </c>
       <c r="C3">
-        <v>19.71859933685019</v>
+        <v>14.37467498741655</v>
       </c>
       <c r="D3">
-        <v>0.3947383778073559</v>
+        <v>0.1946795840814501</v>
       </c>
       <c r="E3">
-        <v>33.63052441273815</v>
+        <v>6.743675143091359</v>
       </c>
       <c r="F3">
-        <v>17.36499705143349</v>
+        <v>9.366207192124389</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -502,16 +502,16 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>553.8869</v>
+        <v>606.2380000000001</v>
       </c>
       <c r="C4">
-        <v>25.2005</v>
+        <v>27.5319</v>
       </c>
       <c r="D4">
-        <v>0.175</v>
+        <v>0.1911</v>
       </c>
       <c r="E4">
-        <v>1.6406</v>
+        <v>1.7924</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -522,19 +522,19 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>241.0892464982152</v>
+        <v>933.9296628156776</v>
       </c>
       <c r="C5">
-        <v>183.3648445338748</v>
+        <v>811.9936650102653</v>
       </c>
       <c r="D5">
-        <v>2.80401386088515</v>
+        <v>6.662731658726979</v>
       </c>
       <c r="E5">
-        <v>146.3351345312151</v>
+        <v>538.9594219695125</v>
       </c>
       <c r="F5">
-        <v>76.83873508275222</v>
+        <v>236.5860920398866</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -542,7 +542,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>163.6246439492933</v>
+        <v>142.1847557754865</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -554,7 +554,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>247.2010724959712</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -562,19 +562,19 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>850.9532402902286</v>
+        <v>1627.759475004623</v>
       </c>
       <c r="C7">
-        <v>1245.891498883344</v>
+        <v>3465.252911727226</v>
       </c>
       <c r="D7">
-        <v>18.39737160868231</v>
+        <v>23.82886154964101</v>
       </c>
       <c r="E7">
-        <v>825.2149865554252</v>
+        <v>1949.992931595298</v>
       </c>
       <c r="F7">
-        <v>241.0487884009725</v>
+        <v>823.297718807123</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -582,19 +582,19 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>914.4263351040289</v>
+        <v>300.9951287114616</v>
       </c>
       <c r="C8">
-        <v>321.3033365112238</v>
+        <v>301.9165135385996</v>
       </c>
       <c r="D8">
-        <v>10.35022479474767</v>
+        <v>3.08323202186992</v>
       </c>
       <c r="E8">
-        <v>596.8902132739015</v>
+        <v>314.6529525585728</v>
       </c>
       <c r="F8">
-        <v>119.9380696475446</v>
+        <v>69.52820048025472</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -602,19 +602,19 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>2605.151771420494</v>
+        <v>342.995812733584</v>
       </c>
       <c r="C9">
-        <v>191.6242730225303</v>
+        <v>167.0885354213826</v>
       </c>
       <c r="D9">
-        <v>5.205566457762343</v>
+        <v>0.7740550608896813</v>
       </c>
       <c r="E9">
-        <v>360.7227649918731</v>
+        <v>86.19759323966218</v>
       </c>
       <c r="F9">
-        <v>84.55364150167945</v>
+        <v>18.52895129563261</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -622,19 +622,19 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>487.6143495846766</v>
+        <v>513.6708915572244</v>
       </c>
       <c r="C10">
-        <v>1029.685324542674</v>
+        <v>600.4577098396339</v>
       </c>
       <c r="D10">
-        <v>2.633391896978738</v>
+        <v>1.766174844054563</v>
       </c>
       <c r="E10">
-        <v>213.1340858055725</v>
+        <v>353.1607737129829</v>
       </c>
       <c r="F10">
-        <v>102.1270373592939</v>
+        <v>189.3270404239644</v>
       </c>
     </row>
   </sheetData>
@@ -672,19 +672,19 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>6.4165290067163</v>
+        <v>4.15025750007553</v>
       </c>
       <c r="C2">
-        <v>3.59968981255922</v>
+        <v>3.692614168981701</v>
       </c>
       <c r="D2">
-        <v>30.49391141196893</v>
+        <v>15.1530819750613</v>
       </c>
       <c r="E2">
-        <v>38.05638718145123</v>
+        <v>15.17554894591368</v>
       </c>
       <c r="F2">
-        <v>16.70675664553934</v>
+        <v>6.07821304265525</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -692,19 +692,19 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>1.152682842842118</v>
+        <v>4.20388947521794</v>
       </c>
       <c r="C3">
-        <v>0.6301002440652889</v>
+        <v>0.256909639357439</v>
       </c>
       <c r="D3">
-        <v>0.6865993461743732</v>
+        <v>0.4525365745394989</v>
       </c>
       <c r="E3">
-        <v>0.9566616918291188</v>
+        <v>0.1759275984607157</v>
       </c>
       <c r="F3">
-        <v>1.626849534819368</v>
+        <v>0.6320825557244859</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -712,16 +712,16 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>8.801518654624497</v>
+        <v>12.43554442232173</v>
       </c>
       <c r="C4">
-        <v>0.8052722675333674</v>
+        <v>0.4920605513527713</v>
       </c>
       <c r="D4">
-        <v>0.3043911925866871</v>
+        <v>0.4442157599757189</v>
       </c>
       <c r="E4">
-        <v>0.04666888783394578</v>
+        <v>0.04675975944719598</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -732,19 +732,19 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>3.831019474342875</v>
+        <v>19.15736692399406</v>
       </c>
       <c r="C5">
-        <v>5.859352955048385</v>
+        <v>14.51225852556157</v>
       </c>
       <c r="D5">
-        <v>4.877240703682467</v>
+        <v>15.48765257611558</v>
       </c>
       <c r="E5">
-        <v>4.162683152262979</v>
+        <v>14.06026161743707</v>
       </c>
       <c r="F5">
-        <v>7.198680198748717</v>
+        <v>15.96611506001948</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -752,7 +752,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>2.600071162679594</v>
+        <v>2.916585312407055</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>23.1591717871165</v>
+        <v>3.043593065840404</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -772,19 +772,19 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>13.52204000244023</v>
+        <v>33.38965102859783</v>
       </c>
       <c r="C7">
-        <v>39.8119827942436</v>
+        <v>61.93231336454421</v>
       </c>
       <c r="D7">
-        <v>31.99998791101294</v>
+        <v>55.390663750026</v>
       </c>
       <c r="E7">
-        <v>23.47425676365123</v>
+        <v>50.87101116108492</v>
       </c>
       <c r="F7">
-        <v>22.58279158455269</v>
+        <v>55.5606037269087</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -792,19 +792,19 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>14.53065679419033</v>
+        <v>6.17420599499508</v>
       </c>
       <c r="C8">
-        <v>10.26712431731235</v>
+        <v>5.395966355911134</v>
       </c>
       <c r="D8">
-        <v>18.00295582179167</v>
+        <v>7.167034305475766</v>
       </c>
       <c r="E8">
-        <v>16.97927734515402</v>
+        <v>8.208600965738023</v>
       </c>
       <c r="F8">
-        <v>11.23646564611041</v>
+        <v>4.692140772994784</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -812,19 +812,19 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>41.39706484173129</v>
+        <v>7.035751084423657</v>
       </c>
       <c r="C9">
-        <v>6.123279809975441</v>
+        <v>2.98626963137933</v>
       </c>
       <c r="D9">
-        <v>9.054449040957346</v>
+        <v>1.799306421434648</v>
       </c>
       <c r="E9">
-        <v>10.2612033759335</v>
+        <v>2.248704934620537</v>
       </c>
       <c r="F9">
-        <v>7.92145555434664</v>
+        <v>1.250434316644834</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -832,19 +832,19 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>7.748417220432767</v>
+        <v>10.53674825796712</v>
       </c>
       <c r="C10">
-        <v>32.90319779926235</v>
+        <v>10.73160776291184</v>
       </c>
       <c r="D10">
-        <v>4.580464571825578</v>
+        <v>4.105508637371505</v>
       </c>
       <c r="E10">
-        <v>6.062861601883969</v>
+        <v>9.213185017297864</v>
       </c>
       <c r="F10">
-        <v>9.567829048766356</v>
+        <v>12.77681745921206</v>
       </c>
     </row>
   </sheetData>
@@ -882,19 +882,19 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>458.6930911920542</v>
+        <v>312.7364552979616</v>
       </c>
       <c r="C2">
-        <v>35.53841050932789</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>48.66995588756266</v>
+        <v>32.70900205828086</v>
       </c>
       <c r="E2">
-        <v>3470.586529513416</v>
+        <v>3578.555880387605</v>
       </c>
       <c r="F2">
-        <v>297.6973802069476</v>
+        <v>160.7074429422057</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -902,19 +902,19 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>331.991672276997</v>
+        <v>1315.502551133894</v>
       </c>
       <c r="C3">
-        <v>6.279137565675085</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>4.136071194704646</v>
+        <v>2.339106679001917</v>
       </c>
       <c r="E3">
-        <v>1.437857678936757</v>
+        <v>1.507900905345171E-05</v>
       </c>
       <c r="F3">
-        <v>21.64942676462103</v>
+        <v>38.22459422835947</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -922,19 +922,19 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>445.095438041007</v>
+        <v>438.0709466916866</v>
       </c>
       <c r="C4">
-        <v>9.568524753400524</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>0.03676523581830246</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>1.139639888322105</v>
+        <v>13.20957408283649</v>
       </c>
       <c r="F4">
-        <v>12.01504278431368</v>
+        <v>10.79791864911858</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -942,19 +942,19 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>69.75966910642957</v>
+        <v>1.163612339471819</v>
       </c>
       <c r="C5">
-        <v>2823.738515028874</v>
+        <v>5567.694119299737</v>
       </c>
       <c r="D5">
-        <v>0.0206292561983788</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0.3942236147172403</v>
+        <v>0.04861143550294392</v>
       </c>
       <c r="F5">
-        <v>261.3777795030268</v>
+        <v>888.8951793916627</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -962,7 +962,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>163.6246439492933</v>
+        <v>142.1847557754865</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>247.2010724959712</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -982,19 +982,19 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>253.8412435167088</v>
+        <v>336.7124480665429</v>
       </c>
       <c r="C7">
-        <v>34.63234277280916</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1.913815935900073</v>
+        <v>3.533601760788727</v>
       </c>
       <c r="E7">
-        <v>0.4411702590983144</v>
+        <v>8.791957842930925</v>
       </c>
       <c r="F7">
-        <v>114.4758920510881</v>
+        <v>95.20090487225919</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1002,19 +1002,19 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>3007.407222435128</v>
+        <v>477.1030916427846</v>
       </c>
       <c r="C8">
-        <v>20.95826533339547</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.04395939992222332</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>4.026475436426869</v>
+        <v>56.99019242517961</v>
       </c>
       <c r="F8">
-        <v>7.204302442250194</v>
+        <v>1.835198498241583</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1022,19 +1022,19 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>1562.670312659033</v>
+        <v>1851.568030356954</v>
       </c>
       <c r="C9">
-        <v>198.72325808781</v>
+        <v>27.5319</v>
       </c>
       <c r="D9">
-        <v>2.670611086329776</v>
+        <v>4.437924827439155</v>
       </c>
       <c r="E9">
-        <v>37.37821145385924</v>
+        <v>175.6142497035181</v>
       </c>
       <c r="F9">
-        <v>105.7794182720509</v>
+        <v>241.0400083120736</v>
       </c>
     </row>
   </sheetData>
@@ -1072,19 +1072,19 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>7.288845067240689</v>
+        <v>6.415051650238419</v>
       </c>
       <c r="C2">
-        <v>1.135616214574239</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>84.65546237575226</v>
+        <v>76.03272740641856</v>
       </c>
       <c r="E2">
-        <v>98.72510877963224</v>
+        <v>93.35662359700562</v>
       </c>
       <c r="F2">
-        <v>27.88994683224768</v>
+        <v>10.84541150704744</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1092,19 +1092,19 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>5.275501003410567</v>
+        <v>26.98443583593097</v>
       </c>
       <c r="C3">
-        <v>0.2006474215061258</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>7.19419224902623</v>
+        <v>5.437300110293651</v>
       </c>
       <c r="E3">
-        <v>0.04090163278037124</v>
+        <v>3.933780607238852E-07</v>
       </c>
       <c r="F3">
-        <v>2.028238746992604</v>
+        <v>2.579603324567582</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1112,19 +1112,19 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>7.072772078570879</v>
+        <v>8.985993483933713</v>
       </c>
       <c r="C4">
-        <v>0.305758521661078</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>0.06394865129407924</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0.0324184603920485</v>
+        <v>0.3446086289407209</v>
       </c>
       <c r="F4">
-        <v>1.125636054333908</v>
+        <v>0.7287022245225295</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1132,19 +1132,19 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>1.108513360725216</v>
+        <v>0.02386876595967841</v>
       </c>
       <c r="C5">
-        <v>90.2314762373209</v>
+        <v>99.50793944864724</v>
       </c>
       <c r="D5">
-        <v>0.03588207940800472</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0.01121417631155158</v>
+        <v>0.001268165047143795</v>
       </c>
       <c r="F5">
-        <v>24.48732457236533</v>
+        <v>59.98747681275888</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1152,7 +1152,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>2.600071162679591</v>
+        <v>2.916585312407057</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>23.15917178711651</v>
+        <v>3.043593065840403</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1172,19 +1172,19 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>4.033654596498653</v>
+        <v>6.906862660341639</v>
       </c>
       <c r="C7">
-        <v>1.106663169169376</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>3.328849800685885</v>
+        <v>8.213927742649414</v>
       </c>
       <c r="E7">
-        <v>0.01254963143821286</v>
+        <v>0.229362772709963</v>
       </c>
       <c r="F7">
-        <v>10.72473845977251</v>
+        <v>6.424674366539687</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1192,19 +1192,19 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>47.78908974073081</v>
+        <v>9.786645987468431</v>
       </c>
       <c r="C8">
-        <v>0.6697132933310586</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0.07646202381554669</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>0.114538053461382</v>
+        <v>1.486748319934617</v>
       </c>
       <c r="F8">
-        <v>0.6749391342917191</v>
+        <v>0.1238491668223681</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1212,19 +1212,19 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>24.83155299014359</v>
+        <v>37.9805563037201</v>
       </c>
       <c r="C9">
-        <v>6.350125142437228</v>
+        <v>0.4920605513527712</v>
       </c>
       <c r="D9">
-        <v>4.64520282001799</v>
+        <v>10.31604474063839</v>
       </c>
       <c r="E9">
-        <v>1.06326926598419</v>
+        <v>4.58138812298388</v>
       </c>
       <c r="F9">
-        <v>9.91000441287974</v>
+        <v>16.26668953190112</v>
       </c>
     </row>
   </sheetData>
@@ -1262,16 +1262,16 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>225.3482</v>
+        <v>246.6378</v>
       </c>
       <c r="C2">
-        <v>25.2005</v>
+        <v>27.5319</v>
       </c>
       <c r="D2">
-        <v>0.175</v>
+        <v>0.1911</v>
       </c>
       <c r="E2">
-        <v>1.6406</v>
+        <v>1.7924</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1282,19 +1282,19 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>329.6664434343356</v>
+        <v>412.9581321090125</v>
       </c>
       <c r="C3">
-        <v>161.1744482061827</v>
+        <v>389.1303615014439</v>
       </c>
       <c r="D3">
-        <v>12.67673942569171</v>
+        <v>5.801537437292059</v>
       </c>
       <c r="E3">
-        <v>128.9869195109789</v>
+        <v>121.941115910655</v>
       </c>
       <c r="F3">
-        <v>28.58799792847372</v>
+        <v>10.64188207745017</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1302,19 +1302,19 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>1321.607677865828</v>
+        <v>642.0608088897418</v>
       </c>
       <c r="C4">
-        <v>542.2471023169179</v>
+        <v>515.1106499279065</v>
       </c>
       <c r="D4">
-        <v>5.69339262304124</v>
+        <v>4.255098843274198</v>
       </c>
       <c r="E4">
-        <v>955.0016334748034</v>
+        <v>997.6042392695101</v>
       </c>
       <c r="F4">
-        <v>177.7856971719516</v>
+        <v>138.2326254470156</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1322,19 +1322,19 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>1153.3814154035</v>
+        <v>1926.864799229101</v>
       </c>
       <c r="C5">
-        <v>391.1795852685976</v>
+        <v>2619.624402800421</v>
       </c>
       <c r="D5">
-        <v>27.65433782604109</v>
+        <v>23.2795048972046</v>
       </c>
       <c r="E5">
-        <v>1040.552167684438</v>
+        <v>878.8013370965516</v>
       </c>
       <c r="F5">
-        <v>196.0860741747706</v>
+        <v>407.2896920167967</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1342,19 +1342,19 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>210.693525046808</v>
+        <v>280.9846273953015</v>
       </c>
       <c r="C6">
-        <v>115.7497431852714</v>
+        <v>1594.52000801272</v>
       </c>
       <c r="D6">
-        <v>3.725600723366846</v>
+        <v>6.318406688230417</v>
       </c>
       <c r="E6">
-        <v>474.967282995189</v>
+        <v>1079.854650892856</v>
       </c>
       <c r="F6">
-        <v>114.5115516957766</v>
+        <v>635.9242052066603</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1362,19 +1362,19 @@
         <v>26</v>
       </c>
       <c r="B7">
-        <v>121.1138394896388</v>
+        <v>92.12503282863821</v>
       </c>
       <c r="C7">
-        <v>48.8980195314555</v>
+        <v>87.65798803431832</v>
       </c>
       <c r="D7">
-        <v>2.579852260294825</v>
+        <v>2.342417493501372</v>
       </c>
       <c r="E7">
-        <v>581.3259584550091</v>
+        <v>575.1196890910694</v>
       </c>
       <c r="F7">
-        <v>47.77597866254364</v>
+        <v>51.24039023150898</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1382,19 +1382,19 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>2931.272191936538</v>
+        <v>1273.410690852991</v>
       </c>
       <c r="C8">
-        <v>1844.98905554287</v>
+        <v>361.6507090229273</v>
       </c>
       <c r="D8">
-        <v>4.986885138000327</v>
+        <v>0.8315699660080151</v>
       </c>
       <c r="E8">
-        <v>332.929545724355</v>
+        <v>178.0970486959332</v>
       </c>
       <c r="F8">
-        <v>502.6530148867536</v>
+        <v>238.4724519144894</v>
       </c>
     </row>
   </sheetData>
@@ -1432,16 +1432,16 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>3.580886975456634</v>
+        <v>5.059193448981592</v>
       </c>
       <c r="C2">
-        <v>0.8052722675333667</v>
+        <v>0.4920605513527712</v>
       </c>
       <c r="D2">
-        <v>0.3043911925866872</v>
+        <v>0.4442157599757188</v>
       </c>
       <c r="E2">
-        <v>0.0466688878339458</v>
+        <v>0.04675975944719601</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -1452,19 +1452,19 @@
         <v>22</v>
       </c>
       <c r="B3">
-        <v>5.238552043189709</v>
+        <v>8.470863252387064</v>
       </c>
       <c r="C3">
-        <v>5.150267390545107</v>
+        <v>6.954685300633217</v>
       </c>
       <c r="D3">
-        <v>22.049644753697</v>
+        <v>13.48578943869323</v>
       </c>
       <c r="E3">
-        <v>3.669191807085256</v>
+        <v>3.181174540674444</v>
       </c>
       <c r="F3">
-        <v>2.678282696714611</v>
+        <v>0.718172028789769</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1472,19 +1472,19 @@
         <v>23</v>
       </c>
       <c r="B4">
-        <v>21.000956388084</v>
+        <v>13.17036495696444</v>
       </c>
       <c r="C4">
-        <v>17.32729722212424</v>
+        <v>9.206252761749461</v>
       </c>
       <c r="D4">
-        <v>9.902963259381542</v>
+        <v>9.891062095430925</v>
       </c>
       <c r="E4">
-        <v>27.16619780194479</v>
+        <v>26.0252924859101</v>
       </c>
       <c r="F4">
-        <v>16.65595323080406</v>
+        <v>9.328688698080935</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1492,19 +1492,19 @@
         <v>24</v>
       </c>
       <c r="B5">
-        <v>18.3277633819668</v>
+        <v>39.52509213645717</v>
       </c>
       <c r="C5">
-        <v>12.49999292244224</v>
+        <v>46.818920160946</v>
       </c>
       <c r="D5">
-        <v>48.10135354893589</v>
+        <v>54.1136732588708</v>
       </c>
       <c r="E5">
-        <v>29.59978812570656</v>
+        <v>22.92598701434332</v>
       </c>
       <c r="F5">
-        <v>18.37043436350299</v>
+        <v>27.48612156121054</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1512,19 +1512,19 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>3.348017422163393</v>
+        <v>5.763737700315372</v>
       </c>
       <c r="C6">
-        <v>3.698738444126442</v>
+        <v>28.49786590412446</v>
       </c>
       <c r="D6">
-        <v>6.480228841642621</v>
+        <v>14.68726231736232</v>
       </c>
       <c r="E6">
-        <v>13.51102941295652</v>
+        <v>28.17102416518956</v>
       </c>
       <c r="F6">
-        <v>10.72807925368117</v>
+        <v>42.91562087288382</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1532,19 +1532,19 @@
         <v>26</v>
       </c>
       <c r="B7">
-        <v>1.924554846126984</v>
+        <v>1.889728024552037</v>
       </c>
       <c r="C7">
-        <v>1.562517373305531</v>
+        <v>1.566656784407952</v>
       </c>
       <c r="D7">
-        <v>4.487338892620584</v>
+        <v>5.4449961646056</v>
       </c>
       <c r="E7">
-        <v>16.53653294532358</v>
+        <v>15.0036031662824</v>
       </c>
       <c r="F7">
-        <v>4.47591948518546</v>
+        <v>3.457979964513902</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1552,19 +1552,19 @@
         <v>27</v>
       </c>
       <c r="B8">
-        <v>46.57926894301248</v>
+        <v>26.12102048034232</v>
       </c>
       <c r="C8">
-        <v>58.95591437992309</v>
+        <v>6.463558536786135</v>
       </c>
       <c r="D8">
-        <v>8.674079511135687</v>
+        <v>1.933000965061398</v>
       </c>
       <c r="E8">
-        <v>9.470591019149367</v>
+        <v>4.646158868152973</v>
       </c>
       <c r="F8">
-        <v>47.09133097011171</v>
+        <v>16.09341687452104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>